<commit_message>
Update backend config value retrieval for new upstream and tariff structure
- Modified `_get_config_value()` to support model and fuel parameters for config lookups

- Added cell_index parameter to retrieve yearly values from config dictionaries

- Updated `_get_cell_value_from_ref()` to pass cell_index for config references

- Enhanced `_execute_single_formula()` to handle single config references with multiple yearly values

Pending adjustments:
- Electricity upstream costs: Conceptual discussion needed on demand types for different electricity variants (grid, off-grid, Electricity & E-Cooking, Electricity (Just Access))

- Tariff structure: Similar refactoring required to align with new hierarchical config format
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="C27" s="13" t="n">
-        <v>289.3223057172883</v>
+        <v>483.6522897428962</v>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>57.86446114345765</v>
+        <v>96.73045794857924</v>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>144.6611528586441</v>
+        <v>241.8261448714481</v>
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>9.258313782953223</v>
+        <v>15.47687327177268</v>
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>57.86446114345765</v>
+        <v>96.73045794857924</v>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>144.6611528586441</v>
+        <v>241.8261448714481</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="C39" s="13" t="n">
-        <v>9.258313782953223</v>
+        <v>15.47687327177268</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
@@ -5363,7 +5363,7 @@
         </is>
       </c>
       <c r="C27" s="13" t="n">
-        <v>272.9424387981718</v>
+        <v>552.568672669074</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
@@ -5592,7 +5592,7 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>68.23560969954296</v>
+        <v>138.1421681672685</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>150.1183413389945</v>
+        <v>303.9127699679907</v>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
@@ -5817,7 +5817,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>8.188273163945155</v>
+        <v>16.57706018007222</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>68.23560969954296</v>
+        <v>138.1421681672685</v>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>150.1183413389945</v>
+        <v>303.9127699679907</v>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
@@ -6271,7 +6271,7 @@
         </is>
       </c>
       <c r="C39" s="13" t="n">
-        <v>8.188273163945155</v>
+        <v>16.57706018007222</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>43.73732570467683</v>
+        <v>43.7241723631853</v>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>21.86866285233842</v>
+        <v>21.86208618159265</v>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
@@ -7970,7 +7970,7 @@
         </is>
       </c>
       <c r="C24" s="13" t="n">
-        <v>2.62423954228061</v>
+        <v>2.623450341791118</v>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adjust decimal rounding logic in design-capital
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -1429,40 +1429,40 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>6255.815858106422</v>
+        <v>132486740.348631</v>
       </c>
       <c r="E12" s="25" t="n">
-        <v>995.2748528889368</v>
+        <v>260707270.7223993</v>
       </c>
       <c r="F12" s="25" t="n">
-        <v>1158.031393407107</v>
+        <v>262419702.007456</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>1362.917594633227</v>
+        <v>254614832.1587506</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>1791.738474540101</v>
+        <v>246182025.5734624</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>1809.770896624647</v>
+        <v>237770947.2312178</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>1800.621998683244</v>
+        <v>250231700.8302397</v>
       </c>
       <c r="K12" s="25" t="n">
-        <v>1789.004074977049</v>
+        <v>264048751.1678632</v>
       </c>
       <c r="L12" s="25" t="n">
-        <v>1758.026355669181</v>
+        <v>257139145.7603923</v>
       </c>
       <c r="M12" s="25" t="n">
-        <v>1727.748915241144</v>
+        <v>248743086.8877178</v>
       </c>
       <c r="N12" s="25" t="n">
-        <v>1688.873353358474</v>
+        <v>240307495.154728</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>1810.726953759539</v>
+        <v>23317882.88694784</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
@@ -1814,7 +1814,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>20946.88607202908</v>
+        <v>9081367717.144072</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>5236.72151800727</v>
+        <v>2270341929.286018</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>11520.78733961599</v>
+        <v>4994752244.429239</v>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
@@ -3052,62 +3052,62 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O11" s="26" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -3128,40 +3128,40 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>77.43450866048723</v>
+        <v>0</v>
       </c>
       <c r="E12" s="25" t="n">
-        <v>93.2408068890778</v>
+        <v>0</v>
       </c>
       <c r="F12" s="25" t="n">
-        <v>128.0757364005578</v>
+        <v>0</v>
       </c>
       <c r="G12" s="25" t="n">
-        <v>185.8346655963578</v>
+        <v>0</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>236.7749771814905</v>
+        <v>0</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>303.4599333508003</v>
+        <v>0</v>
       </c>
       <c r="J12" s="25" t="n">
-        <v>345.7448629505327</v>
+        <v>0</v>
       </c>
       <c r="K12" s="25" t="n">
-        <v>423.9007959863739</v>
+        <v>0</v>
       </c>
       <c r="L12" s="25" t="n">
-        <v>432.3978128742861</v>
+        <v>0</v>
       </c>
       <c r="M12" s="25" t="n">
-        <v>437.010398470347</v>
+        <v>0</v>
       </c>
       <c r="N12" s="25" t="n">
-        <v>422.9834251400963</v>
+        <v>0</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>419.1103869175019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
@@ -4844,17 +4844,17 @@
       </c>
       <c r="M11" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N11" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O11" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
     </row>
@@ -4875,40 +4875,40 @@
         </is>
       </c>
       <c r="D12" s="39" t="n">
-        <v>6409.015315803753</v>
+        <v>50266702.88239282</v>
       </c>
       <c r="E12" s="39" t="n">
-        <v>1182.167626561949</v>
+        <v>175394835.7352284</v>
       </c>
       <c r="F12" s="39" t="n">
-        <v>1431.044029517446</v>
+        <v>180025441.3453405</v>
       </c>
       <c r="G12" s="39" t="n">
-        <v>1679.319219959062</v>
+        <v>174664900.8487673</v>
       </c>
       <c r="H12" s="39" t="n">
-        <v>2228.944294722068</v>
+        <v>168537337.1575918</v>
       </c>
       <c r="I12" s="39" t="n">
-        <v>2280.95442146801</v>
+        <v>162397328.7399543</v>
       </c>
       <c r="J12" s="39" t="n">
-        <v>2315.813491932639</v>
+        <v>219476630.2792167</v>
       </c>
       <c r="K12" s="39" t="n">
-        <v>2366.844027442179</v>
+        <v>280931435.4419159</v>
       </c>
       <c r="L12" s="39" t="n">
-        <v>75.42130482923767</v>
+        <v>279335396.8377594</v>
       </c>
       <c r="M12" s="39" t="n">
-        <v>0</v>
+        <v>272554461.4585249</v>
       </c>
       <c r="N12" s="39" t="n">
-        <v>0</v>
+        <v>265404697.5498739</v>
       </c>
       <c r="O12" s="39" t="n">
-        <v>0</v>
+        <v>60504314.41676617</v>
       </c>
     </row>
     <row r="13">
@@ -5260,7 +5260,7 @@
         </is>
       </c>
       <c r="C18" s="32" t="n">
-        <v>25929.02996132894</v>
+        <v>7012041909.345428</v>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="C21" s="33" t="n">
-        <v>5185.805992265789</v>
+        <v>1402408381.869086</v>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
@@ -5564,7 +5564,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>12964.51498066447</v>
+        <v>3506020954.672714</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix GRANTS realisation % capex calculation
- Add "direction": "forward" with "from_start": true to SUM_RANGE for summing from index 0

- Implement SET_VALUES operation to zero out values after realisation period

- Enable in-memory array modification for CACHED:: sources and temp results
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -6,9 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Electricity (Low access)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LPG" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Electricity &amp; E-Cooking" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Electricity (Low access)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -645,9 +645,9 @@
   <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30.6328125" customWidth="1" min="1" max="1"/>
-    <col width="12.90625" customWidth="1" min="3" max="3"/>
-    <col width="9.36328125" customWidth="1" min="4" max="4"/>
+    <col width="39.36328125" customWidth="1" min="1" max="1"/>
+    <col width="22.36328125" customWidth="1" min="2" max="2"/>
+    <col width="13.6328125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C2" s="32" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" s="29" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="C4" s="32" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="29" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C5" s="32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
@@ -990,10 +990,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C6" s="33" t="n">
+        <v>1003</v>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
@@ -1359,12 +1357,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>FFSS - Outputs</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
@@ -1374,40 +1372,40 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="40" t="n">
         <v>2023</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="40" t="n">
         <v>2024</v>
       </c>
-      <c r="F11" s="38" t="n">
+      <c r="F11" s="40" t="n">
         <v>2025</v>
       </c>
-      <c r="G11" s="38" t="n">
+      <c r="G11" s="40" t="n">
         <v>2026</v>
       </c>
-      <c r="H11" s="38" t="n">
+      <c r="H11" s="40" t="n">
         <v>2027</v>
       </c>
-      <c r="I11" s="38" t="n">
+      <c r="I11" s="40" t="n">
         <v>2028</v>
       </c>
-      <c r="J11" s="38" t="n">
+      <c r="J11" s="40" t="n">
         <v>2029</v>
       </c>
-      <c r="K11" s="38" t="n">
+      <c r="K11" s="40" t="n">
         <v>2030</v>
       </c>
-      <c r="L11" s="38" t="n">
+      <c r="L11" s="40" t="n">
         <v>2031</v>
       </c>
-      <c r="M11" s="38" t="n">
+      <c r="M11" s="40" t="n">
         <v>2032</v>
       </c>
-      <c r="N11" s="38" t="n">
+      <c r="N11" s="40" t="n">
         <v>2033</v>
       </c>
-      <c r="O11" s="38" t="n">
+      <c r="O11" s="40" t="n">
         <v>2034</v>
       </c>
     </row>
@@ -1542,77 +1540,77 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="36" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="33" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1817,62 +1815,62 @@
           <t>Amount</t>
         </is>
       </c>
-      <c r="D18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="41" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1890,7 +1888,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1046.78135238923</v>
+        <v>1156.678041401294</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2033,7 +2031,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t xml:space="preserve">Total </t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -2119,7 +2117,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>261.6953380973075</v>
+        <v>578.339020700647</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2194,7 +2192,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>575.7297438140764</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -2271,62 +2269,62 @@
       <c r="C24" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2346,62 +2344,62 @@
       <c r="C25" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2738,7 +2736,7 @@
         </is>
       </c>
       <c r="C5" s="32" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
@@ -4016,7 +4014,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>780.5151909790567</v>
+        <v>780.5151909790565</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -4243,9 +4241,9 @@
   <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39.36328125" customWidth="1" min="1" max="1"/>
-    <col width="22.36328125" customWidth="1" min="2" max="2"/>
-    <col width="13.6328125" customWidth="1" min="3" max="3"/>
+    <col width="30.6328125" customWidth="1" min="1" max="1"/>
+    <col width="12.90625" customWidth="1" min="3" max="3"/>
+    <col width="9.36328125" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4289,7 +4287,7 @@
         </is>
       </c>
       <c r="C2" s="32" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
@@ -4386,7 +4384,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="H3" s="29" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4439,7 +4437,7 @@
         </is>
       </c>
       <c r="C4" s="32" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
@@ -4461,7 +4459,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="29" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4514,7 +4512,7 @@
         </is>
       </c>
       <c r="C5" s="32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
@@ -4588,8 +4586,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="33" t="n">
-        <v>1003</v>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
@@ -4955,12 +4955,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>FFSS - Outputs</t>
         </is>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
@@ -4970,40 +4970,40 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="38" t="n">
         <v>2023</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="38" t="n">
         <v>2024</v>
       </c>
-      <c r="F11" s="40" t="n">
+      <c r="F11" s="38" t="n">
         <v>2025</v>
       </c>
-      <c r="G11" s="40" t="n">
+      <c r="G11" s="38" t="n">
         <v>2026</v>
       </c>
-      <c r="H11" s="40" t="n">
+      <c r="H11" s="38" t="n">
         <v>2027</v>
       </c>
-      <c r="I11" s="40" t="n">
+      <c r="I11" s="38" t="n">
         <v>2028</v>
       </c>
-      <c r="J11" s="40" t="n">
+      <c r="J11" s="38" t="n">
         <v>2029</v>
       </c>
-      <c r="K11" s="40" t="n">
+      <c r="K11" s="38" t="n">
         <v>2030</v>
       </c>
-      <c r="L11" s="40" t="n">
+      <c r="L11" s="38" t="n">
         <v>2031</v>
       </c>
-      <c r="M11" s="40" t="n">
+      <c r="M11" s="38" t="n">
         <v>2032</v>
       </c>
-      <c r="N11" s="40" t="n">
+      <c r="N11" s="38" t="n">
         <v>2033</v>
       </c>
-      <c r="O11" s="40" t="n">
+      <c r="O11" s="38" t="n">
         <v>2034</v>
       </c>
     </row>
@@ -5138,77 +5138,77 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="33" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="36" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5413,62 +5413,62 @@
           <t>Amount</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="14" t="inlineStr">
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="41" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1156.678041401294</v>
+        <v>1046.78135238923</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total </t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>578.339020700647</v>
+        <v>261.6953380973075</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0</v>
+        <v>575.7297438140765</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5867,62 +5867,62 @@
       <c r="C24" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" s="14" t="inlineStr">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5942,62 +5942,62 @@
       <c r="C25" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Resolved grants calculation and cache logic
TODO: Fix Electricity (Only E-Cooking) sheet calculation
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -6,9 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LPG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Electricity &amp; E-Cooking" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Electricity (Low access)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Electricity &amp; E-Cooking" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Electricity (Low access)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -645,9 +645,7 @@
   <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39.36328125" customWidth="1" min="1" max="1"/>
-    <col width="22.36328125" customWidth="1" min="2" max="2"/>
-    <col width="13.6328125" customWidth="1" min="3" max="3"/>
+    <col width="46.54296875" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,18 +664,66 @@
           <t>Amount</t>
         </is>
       </c>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="14" t="n"/>
-      <c r="L1" s="14" t="n"/>
-      <c r="M1" s="14" t="n"/>
-      <c r="N1" s="14" t="n"/>
-      <c r="O1" s="14" t="n"/>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
@@ -691,7 +737,7 @@
         </is>
       </c>
       <c r="C2" s="32" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
@@ -766,7 +812,7 @@
         </is>
       </c>
       <c r="C3" s="33" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
@@ -788,7 +834,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="H3" s="29" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -841,7 +887,7 @@
         </is>
       </c>
       <c r="C4" s="32" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
@@ -863,7 +909,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="29" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -916,7 +962,7 @@
         </is>
       </c>
       <c r="C5" s="32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
@@ -990,8 +1036,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C6" s="33" t="n">
-        <v>1003</v>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
@@ -1357,12 +1405,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>FFSS - Outputs</t>
         </is>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
@@ -1372,40 +1420,40 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="38" t="n">
         <v>2023</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="38" t="n">
         <v>2024</v>
       </c>
-      <c r="F11" s="40" t="n">
+      <c r="F11" s="38" t="n">
         <v>2025</v>
       </c>
-      <c r="G11" s="40" t="n">
+      <c r="G11" s="38" t="n">
         <v>2026</v>
       </c>
-      <c r="H11" s="40" t="n">
+      <c r="H11" s="38" t="n">
         <v>2027</v>
       </c>
-      <c r="I11" s="40" t="n">
+      <c r="I11" s="38" t="n">
         <v>2028</v>
       </c>
-      <c r="J11" s="40" t="n">
+      <c r="J11" s="38" t="n">
         <v>2029</v>
       </c>
-      <c r="K11" s="40" t="n">
+      <c r="K11" s="38" t="n">
         <v>2030</v>
       </c>
-      <c r="L11" s="40" t="n">
+      <c r="L11" s="38" t="n">
         <v>2031</v>
       </c>
-      <c r="M11" s="40" t="n">
+      <c r="M11" s="38" t="n">
         <v>2032</v>
       </c>
-      <c r="N11" s="40" t="n">
+      <c r="N11" s="38" t="n">
         <v>2033</v>
       </c>
-      <c r="O11" s="40" t="n">
+      <c r="O11" s="38" t="n">
         <v>2034</v>
       </c>
     </row>
@@ -1432,52 +1480,52 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
@@ -1506,111 +1554,111 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>0</v>
+        <v>239.0483893324428</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>0</v>
+        <v>209.6616710419028</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>0</v>
+        <v>193.9013568647863</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>0</v>
+        <v>166.9988372288568</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>0</v>
+        <v>138.583878118821</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0</v>
+        <v>151.2406658118593</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>0</v>
+        <v>151.6276896610999</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>0</v>
+        <v>108.0707718935789</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>0</v>
+        <v>65.39705560395237</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>0</v>
+        <v>24.04768999445366</v>
       </c>
       <c r="O13" s="39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="33" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="36" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1888,7 +1936,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1156.678041401294</v>
+        <v>1643.141631292455</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2031,7 +2079,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total </t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -2117,7 +2165,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>578.339020700647</v>
+        <v>328.628326258491</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2192,7 +2240,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0</v>
+        <v>821.5708156462275</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -2342,7 +2390,7 @@
         </is>
       </c>
       <c r="C25" s="32" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
@@ -2411,1828 +2459,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46.54296875" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t>Division</t>
-        </is>
-      </c>
-      <c r="B1" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C1" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H1" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="30" t="inlineStr">
-        <is>
-          <t>1. Equity</t>
-        </is>
-      </c>
-      <c r="B2" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C2" s="32" t="n">
-        <v>20</v>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H2" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="32" t="inlineStr">
-        <is>
-          <t>Cost of Equity</t>
-        </is>
-      </c>
-      <c r="B3" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H3" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="30" t="inlineStr">
-        <is>
-          <t>2. Grants</t>
-        </is>
-      </c>
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C4" s="32" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="32" t="inlineStr">
-        <is>
-          <t>Years realisation</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C5" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>3. Debt</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="32" t="inlineStr">
-        <is>
-          <t>Cost of Debt</t>
-        </is>
-      </c>
-      <c r="B7" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="32" t="inlineStr">
-        <is>
-          <t>Grace period</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="32" t="inlineStr">
-        <is>
-          <t>Amortization period</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>25</v>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B10" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>FFSS - Outputs</t>
-        </is>
-      </c>
-      <c r="B11" s="37" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C11" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D11" s="38" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E11" s="38" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F11" s="38" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G11" s="38" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H11" s="38" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I11" s="38" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J11" s="38" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K11" s="38" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L11" s="38" t="n">
-        <v>2031</v>
-      </c>
-      <c r="M11" s="38" t="n">
-        <v>2032</v>
-      </c>
-      <c r="N11" s="38" t="n">
-        <v>2033</v>
-      </c>
-      <c r="O11" s="38" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>Calculated debt requirement</t>
-        </is>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>Annual debt needs</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="I12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="N12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>Calculated debt variation</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>How much to increase</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="39" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>FFSS - Inputs</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D15" s="40" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E15" s="40" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F15" s="40" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G15" s="40" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H15" s="40" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I15" s="40" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J15" s="40" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K15" s="40" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L15" s="40" t="n">
-        <v>2031</v>
-      </c>
-      <c r="M15" s="40" t="n">
-        <v>2032</v>
-      </c>
-      <c r="N15" s="40" t="n">
-        <v>2033</v>
-      </c>
-      <c r="O15" s="40" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>User-defined debt increase</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>Debt increase</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Financiation</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
-        <is>
-          <t>How much to be financed</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C19" s="32" t="n">
-        <v>1561.030381958113</v>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C21" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="B22" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="n">
-        <v>312.2060763916226</v>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Grants</t>
-        </is>
-      </c>
-      <c r="B23" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="n">
-        <v>780.5151909790565</v>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="33" t="inlineStr">
-        <is>
-          <t>Debt</t>
-        </is>
-      </c>
-      <c r="B24" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>WACC</t>
-        </is>
-      </c>
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C25" s="32" t="n">
-        <v>16</v>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5030,52 +3256,52 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
@@ -5104,34 +3330,34 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>0</v>
+        <v>171.0021568857184</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>0</v>
+        <v>150.6157230085008</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>0</v>
+        <v>142.419382512402</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>0</v>
+        <v>124.2558018835478</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>0</v>
+        <v>104.8227788471428</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0</v>
+        <v>93.64588923075212</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>0</v>
+        <v>78.78006578582284</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>0</v>
+        <v>54.09524368810372</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>0</v>
+        <v>29.96587834175676</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>0</v>
+        <v>6.755942096130582</v>
       </c>
       <c r="O13" s="39" t="n">
         <v>0</v>
@@ -5486,7 +3712,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1046.78135238923</v>
+        <v>1110.343595730213</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5715,7 +3941,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>261.6953380973075</v>
+        <v>277.5858989325532</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +4016,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>575.7297438140765</v>
+        <v>610.6889776516169</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5998,6 +4224,1780 @@
         </is>
       </c>
       <c r="O25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39.36328125" customWidth="1" min="1" max="1"/>
+    <col width="22.36328125" customWidth="1" min="2" max="2"/>
+    <col width="13.6328125" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="14" t="n"/>
+      <c r="L1" s="14" t="n"/>
+      <c r="M1" s="14" t="n"/>
+      <c r="N1" s="14" t="n"/>
+      <c r="O1" s="14" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>1. Equity</t>
+        </is>
+      </c>
+      <c r="B2" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Cost of Equity</t>
+        </is>
+      </c>
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C3" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>2. Grants</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>Years realisation</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>3. Debt</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>1003</v>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Cost of Debt</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Grace period</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>Amortization period</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>FFSS - Outputs</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H11" s="40" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I11" s="40" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J11" s="40" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K11" s="40" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L11" s="40" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M11" s="40" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N11" s="40" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O11" s="40" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Calculated debt requirement</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Annual debt needs</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="G12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="H12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="I12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="J12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="K12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="L12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="M12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="N12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="O12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Calculated debt variation</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>How much to increase</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="39" t="n">
+        <v>41.88050433879165</v>
+      </c>
+      <c r="F13" s="39" t="n">
+        <v>58.126533642865</v>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>74.46520162336132</v>
+      </c>
+      <c r="H13" s="39" t="n">
+        <v>88.86404943358382</v>
+      </c>
+      <c r="I13" s="39" t="n">
+        <v>105.4145733742163</v>
+      </c>
+      <c r="J13" s="39" t="n">
+        <v>118.3193406935254</v>
+      </c>
+      <c r="K13" s="39" t="n">
+        <v>127.7327592582115</v>
+      </c>
+      <c r="L13" s="39" t="n">
+        <v>125.3261715029091</v>
+      </c>
+      <c r="M13" s="39" t="n">
+        <v>129.8283674257615</v>
+      </c>
+      <c r="N13" s="39" t="n">
+        <v>130.7617291779292</v>
+      </c>
+      <c r="O13" s="39" t="n">
+        <v>135.098786157287</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>FFSS - Inputs</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E15" s="40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F15" s="40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G15" s="40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H15" s="40" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I15" s="40" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J15" s="40" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K15" s="40" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L15" s="40" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M15" s="40" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N15" s="40" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O15" s="40" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>User-defined debt increase</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Debt increase</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Financiation</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>How much to be financed</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n">
+        <v>1167.034124287851</v>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total </t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="n">
+        <v>583.5170621439256</v>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>Grants</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>233.4068248575703</v>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Correct debt repayment calculation logic
- Fix A164, first non-zero debt year

- Adjust index matching behavior

- Ensure grace period addition with correct base year

- Validate condition evaluation for debt repayment start year
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -6,9 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Electricity &amp; E-Cooking" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Electricity (Low access)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Electricity (Low access)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LPG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Electricity &amp; E-Cooking" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -645,1828 +645,6 @@
   <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46.54296875" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t>Division</t>
-        </is>
-      </c>
-      <c r="B1" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C1" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H1" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O1" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="30" t="inlineStr">
-        <is>
-          <t>1. Equity</t>
-        </is>
-      </c>
-      <c r="B2" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C2" s="32" t="n">
-        <v>20</v>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H2" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O2" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="32" t="inlineStr">
-        <is>
-          <t>Cost of Equity</t>
-        </is>
-      </c>
-      <c r="B3" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H3" s="29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="30" t="inlineStr">
-        <is>
-          <t>2. Grants</t>
-        </is>
-      </c>
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C4" s="32" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="32" t="inlineStr">
-        <is>
-          <t>Years realisation</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C5" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>3. Debt</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="32" t="inlineStr">
-        <is>
-          <t>Cost of Debt</t>
-        </is>
-      </c>
-      <c r="B7" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O7" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="32" t="inlineStr">
-        <is>
-          <t>Grace period</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="32" t="inlineStr">
-        <is>
-          <t>Amortization period</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>25</v>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B10" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>FFSS - Outputs</t>
-        </is>
-      </c>
-      <c r="B11" s="37" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C11" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D11" s="38" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E11" s="38" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F11" s="38" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G11" s="38" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H11" s="38" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I11" s="38" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J11" s="38" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K11" s="38" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L11" s="38" t="n">
-        <v>2031</v>
-      </c>
-      <c r="M11" s="38" t="n">
-        <v>2032</v>
-      </c>
-      <c r="N11" s="38" t="n">
-        <v>2033</v>
-      </c>
-      <c r="O11" s="38" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>Calculated debt requirement</t>
-        </is>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>Annual debt needs</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E12" s="39" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="G12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="H12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="I12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="J12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="K12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="L12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="M12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="N12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="O12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>Calculated debt variation</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>How much to increase</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="39" t="n">
-        <v>99.96953420761</v>
-      </c>
-      <c r="G13" s="39" t="n">
-        <v>204.3095418366817</v>
-      </c>
-      <c r="H13" s="39" t="n">
-        <v>282.6418390654526</v>
-      </c>
-      <c r="I13" s="39" t="n">
-        <v>333.4462325268448</v>
-      </c>
-      <c r="J13" s="39" t="n">
-        <v>387.838575985439</v>
-      </c>
-      <c r="K13" s="39" t="n">
-        <v>433.687834140141</v>
-      </c>
-      <c r="L13" s="39" t="n">
-        <v>541.7586060337198</v>
-      </c>
-      <c r="M13" s="39" t="n">
-        <v>607.1556616376722</v>
-      </c>
-      <c r="N13" s="39" t="n">
-        <v>631.2033516321258</v>
-      </c>
-      <c r="O13" s="39" t="n">
-        <v>631.2033516321258</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>FFSS - Inputs</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D15" s="40" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E15" s="40" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F15" s="40" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G15" s="40" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H15" s="40" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I15" s="40" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J15" s="40" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K15" s="40" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L15" s="40" t="n">
-        <v>2031</v>
-      </c>
-      <c r="M15" s="40" t="n">
-        <v>2032</v>
-      </c>
-      <c r="N15" s="40" t="n">
-        <v>2033</v>
-      </c>
-      <c r="O15" s="40" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>User-defined debt increase</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>Debt increase</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Financiation</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
-        <is>
-          <t>How much to be financed</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C19" s="32" t="n">
-        <v>1445.62611380047</v>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O19" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O20" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C21" s="28" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O21" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="B22" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="n">
-        <v>289.1252227600941</v>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O22" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Grants</t>
-        </is>
-      </c>
-      <c r="B23" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="n">
-        <v>722.8130569002351</v>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="33" t="inlineStr">
-        <is>
-          <t>Debt</t>
-        </is>
-      </c>
-      <c r="B24" s="34" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>WACC</t>
-        </is>
-      </c>
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C25" s="32" t="n">
-        <v>16</v>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
     <col width="30.6328125" customWidth="1" min="1" max="1"/>
     <col width="12.90625" customWidth="1" min="3" max="3"/>
     <col width="9.36328125" customWidth="1" min="4" max="4"/>
@@ -3342,7 +1520,7 @@
         <v>139.4228455577152</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>174.5037518729916</v>
+        <v>174.5037518729917</v>
       </c>
       <c r="J13" s="39" t="n">
         <v>197.2210512141922</v>
@@ -3351,16 +1529,16 @@
         <v>203.9053063208444</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>258.0005500089481</v>
+        <v>258.0005500089482</v>
       </c>
       <c r="M13" s="39" t="n">
         <v>287.9664283507049</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>294.7223704468354</v>
+        <v>294.7223704468355</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>294.7223704468354</v>
+        <v>294.7223704468355</v>
       </c>
     </row>
     <row r="14">
@@ -4234,7 +2412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5104,7 +3282,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>9.78588892032105</v>
+        <v>9.785888920321048</v>
       </c>
       <c r="F13" s="39" t="n">
         <v>46.1742513621563</v>
@@ -5128,7 +3306,7 @@
         <v>429.5676106826317</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>502.5390211603806</v>
+        <v>502.5390211603807</v>
       </c>
       <c r="N13" s="39" t="n">
         <v>582.4192870297329</v>
@@ -5941,6 +4119,1828 @@
       </c>
       <c r="C25" s="32" t="n">
         <v>12</v>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46.54296875" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>1. Equity</t>
+        </is>
+      </c>
+      <c r="B2" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Cost of Equity</t>
+        </is>
+      </c>
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C3" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>2. Grants</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>Years realisation</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>3. Debt</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Cost of Debt</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Grace period</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>Amortization period</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>FFSS - Outputs</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G11" s="38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H11" s="38" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I11" s="38" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J11" s="38" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K11" s="38" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L11" s="38" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M11" s="38" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N11" s="38" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O11" s="38" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Calculated debt requirement</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Annual debt needs</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="G12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="H12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="I12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="J12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="K12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="L12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="M12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="N12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+      <c r="O12" s="39" t="inlineStr">
+        <is>
+          <t>increase debt</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Calculated debt variation</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>How much to increase</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="39" t="n">
+        <v>105.2311008423658</v>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>210.4384550677187</v>
+      </c>
+      <c r="H13" s="39" t="n">
+        <v>289.6294332155398</v>
+      </c>
+      <c r="I13" s="39" t="n">
+        <v>224.7399170104369</v>
+      </c>
+      <c r="J13" s="39" t="n">
+        <v>131.5901769192128</v>
+      </c>
+      <c r="K13" s="39" t="n">
+        <v>29.48783414014113</v>
+      </c>
+      <c r="L13" s="39" t="n">
+        <v>27.51060603372002</v>
+      </c>
+      <c r="M13" s="39" t="n">
+        <v>34.62766163767236</v>
+      </c>
+      <c r="N13" s="39" t="n">
+        <v>39.85935163212601</v>
+      </c>
+      <c r="O13" s="39" t="n">
+        <v>39.85935163212601</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>FFSS - Inputs</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E15" s="40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F15" s="40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G15" s="40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H15" s="40" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I15" s="40" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J15" s="40" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K15" s="40" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L15" s="40" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M15" s="40" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N15" s="40" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O15" s="40" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>User-defined debt increase</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Debt increase</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="J16" s="33" t="n">
+        <v>160</v>
+      </c>
+      <c r="K16" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="L16" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="M16" s="33" t="n">
+        <v>95</v>
+      </c>
+      <c r="N16" s="33" t="n">
+        <v>60</v>
+      </c>
+      <c r="O16" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Financiation</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>How much to be financed</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n">
+        <v>1431.62611380047</v>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="n">
+        <v>286.3252227600941</v>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>Grants</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>715.8130569002352</v>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>745</v>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n">
+        <v>8.602915325212981</v>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Iterative circular formula resolution
- Split formulas into non-circular, circular and post-circular groups

- Circular formulas iterate until convergence (tol=1e-8, max 50 iter)

- Add circular and post_circular flags to formulas_map.json

- Covers ACoSt → subsidies → revenues → taxes → ACoSt cycle

- Refactor WACC and Annual Cost of Service formula sources
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -1439,52 +1439,52 @@
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -1511,34 +1511,34 @@
         <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>14.3518914887853</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>85.61377279657357</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>139.4228455577152</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>174.5037518729917</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>197.2210512141922</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>203.9053063208444</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>258.0005500089482</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>287.9664283507049</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>294.7223704468355</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>294.7223704468355</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1019.526531604222</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>254.8816329010555</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>560.739592382322</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -3208,57 +3208,57 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -3282,37 +3282,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>9.785888920321048</v>
+        <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>46.1742513621563</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>91.90205973843209</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>149.7391847266321</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>216.3111720417033</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>292.7414325310211</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>358.5648409233147</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>429.5676106826317</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>502.5390211603807</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>582.4192870297329</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>664.5212310339712</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>32.61962973440349</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>16.30981486720174</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>6.523925946880698</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5035,52 +5035,52 @@
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -5107,34 +5107,34 @@
         <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>105.2311008423658</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>210.4384550677187</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>289.6294332155398</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>224.7399170104369</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>131.5901769192128</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>29.48783414014113</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>27.51060603372002</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>34.62766163767236</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>39.85935163212601</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>39.85935163212601</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1431.62611380047</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>286.3252227600941</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>715.8130569002352</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="C25" s="32" t="n">
-        <v>8.602915325212981</v>
+        <v>16</v>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Correct ACoS formulas and ΔWC handling
- Fixed absolute value logic for ΔWC
- Removed incorrect boolean usage in conditional
- Ensured consistent cost aggregation
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -1434,57 +1434,57 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
     </row>
@@ -1508,37 +1508,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>0</v>
+        <v>143.0070847717835</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>0</v>
+        <v>262.907360694831</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>0</v>
+        <v>351.9228306000692</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>0</v>
+        <v>423.3081564013346</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>0</v>
+        <v>475.7894560972919</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0</v>
+        <v>516.2032313318125</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>0</v>
+        <v>540.8751805076691</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>0</v>
+        <v>594.9704241957729</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>0</v>
+        <v>624.9363025375296</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>0</v>
+        <v>631.6922446336603</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>0</v>
+        <v>631.6922446336603</v>
       </c>
     </row>
     <row r="14">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>0</v>
+        <v>1153.001293682047</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0</v>
+        <v>288.2503234205118</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0</v>
+        <v>634.150711525126</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -3208,57 +3208,57 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
     </row>
@@ -3282,37 +3282,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>0</v>
+        <v>31.54124605794365</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>0</v>
+        <v>88.18035638441954</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>0</v>
+        <v>159.3498724636429</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>0</v>
+        <v>241.7705939896951</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>0</v>
+        <v>332.1781496850998</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0</v>
+        <v>421.3851176241964</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>0</v>
+        <v>501.9694332449563</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>0</v>
+        <v>573.1493957344226</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>0</v>
+        <v>646.1208062121715</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>0</v>
+        <v>726.0010720815237</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>0</v>
+        <v>808.103016085762</v>
       </c>
     </row>
     <row r="14">
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>0</v>
+        <v>54.37498687202609</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0</v>
+        <v>27.18749343601305</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0</v>
+        <v>10.87499737440522</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5025,62 +5025,62 @@
       </c>
       <c r="D12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>increase debt</t>
         </is>
       </c>
     </row>
@@ -5101,40 +5101,40 @@
         </is>
       </c>
       <c r="D13" s="39" t="n">
-        <v>0</v>
+        <v>45.87079008676903</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>0</v>
+        <v>248.2483952969826</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>0</v>
+        <v>408.8713205165426</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>0</v>
+        <v>554.2245436026492</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>0</v>
+        <v>673.1602924306418</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>0</v>
+        <v>647.6179244071388</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0</v>
+        <v>597.8804383937903</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>0</v>
+        <v>543.1932705287948</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>0</v>
+        <v>541.2160424223737</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>0</v>
+        <v>548.3330980263261</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>0</v>
+        <v>553.5647880207797</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>0</v>
+        <v>553.5647880207797</v>
       </c>
     </row>
     <row r="14">
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>0</v>
+        <v>1491.730283380381</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0</v>
+        <v>298.3460566760763</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0</v>
+        <v>745.8651416901907</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add notebooks folder, fix excel_editor Arrow type error
- Add notebooks/ folder for AI lab exploration (linking to platform backend + sensitivity analysis and Monte Carlo simulation of financial planning parameters)
- Fix pyarrow type conversion error in excel_editor.py (mixed types in year columns)
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -1508,37 +1508,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>143.0070847717835</v>
+        <v>32.76053524292911</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>262.907360694831</v>
+        <v>129.4325986170056</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>351.9228306000692</v>
+        <v>207.0727386268931</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>423.3081564013346</v>
+        <v>243.9802655280589</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>475.7894560972919</v>
+        <v>241.6601110204685</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>516.2032313318125</v>
+        <v>207.1396449035606</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>540.8751805076691</v>
+        <v>153.0315282935943</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>594.9704241957729</v>
+        <v>153.0315282935943</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>624.9363025375296</v>
+        <v>153.0315282935943</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>631.6922446336603</v>
+        <v>153.0315282935943</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>631.6922446336603</v>
+        <v>153.0315282935943</v>
       </c>
     </row>
     <row r="14">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1153.001293682047</v>
+        <v>765.1576414679723</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>288.2503234205118</v>
+        <v>191.2894103669931</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>634.150711525126</v>
+        <v>420.8367028073848</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -3282,37 +3282,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>31.54124605794365</v>
+        <v>9.785888920321048</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>88.18035638441954</v>
+        <v>46.1742513621563</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>159.3498724636429</v>
+        <v>91.90205973843209</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>241.7705939896951</v>
+        <v>149.7391847266321</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>332.1781496850998</v>
+        <v>216.3111720417033</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>421.3851176241964</v>
+        <v>292.7414325310211</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>501.9694332449563</v>
+        <v>358.5648409233147</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>573.1493957344226</v>
+        <v>429.5676106826317</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>646.1208062121715</v>
+        <v>489.5432484211076</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>726.0010720815237</v>
+        <v>536.5221375252406</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>808.103016085762</v>
+        <v>568.4393062135854</v>
       </c>
     </row>
     <row r="14">
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>54.37498687202609</v>
+        <v>32.61962973440349</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>27.18749343601305</v>
+        <v>16.30981486720174</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>10.87499737440522</v>
+        <v>6.523925946880698</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5025,62 +5025,62 @@
       </c>
       <c r="D12" s="39" t="inlineStr">
         <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="E12" s="39" t="inlineStr">
+      <c r="F12" s="39" t="inlineStr">
         <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
+      <c r="G12" s="39" t="inlineStr">
         <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="G12" s="39" t="inlineStr">
+      <c r="H12" s="39" t="inlineStr">
         <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="H12" s="39" t="inlineStr">
+      <c r="I12" s="39" t="inlineStr">
         <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="I12" s="39" t="inlineStr">
+      <c r="J12" s="39" t="inlineStr">
         <is>
           <t>increase debt</t>
         </is>
       </c>
-      <c r="J12" s="39" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -5101,40 +5101,40 @@
         </is>
       </c>
       <c r="D13" s="39" t="n">
-        <v>45.87079008676903</v>
+        <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>248.2483952969826</v>
+        <v>188.1442257170714</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>408.8713205165426</v>
+        <v>321.726759825858</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>554.2245436026492</v>
+        <v>389.0185416170291</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>673.1602924306418</v>
+        <v>392.5065467157357</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>647.6179244071388</v>
+        <v>224.9243005734117</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>597.8804383937903</v>
+        <v>12.42614874820384</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>543.1932705287948</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>541.2160424223737</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>548.3330980263261</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>553.5647880207797</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>553.5647880207797</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>1491.730283380381</v>
+        <v>783.624304073695</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>298.3460566760763</v>
+        <v>156.724860814739</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>745.8651416901907</v>
+        <v>391.8121520368475</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Restore working baseline config and remove unused ethanol fuel
Replace config.json, formulas_map.json, requirements.txt, excel_editor.py,
and the Rwanda scenario Excel files with a verified working baseline that
does not exhibit the PyArrow serialization error or the design-capital
recalculation issues found in the previous setup.

Also removes the ethanol fuel entry, which was present but unused in the
analysis and had no effect on results.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-CleanStep.xlsx
+++ b/backend/Rwanda/design-capital-CleanStep.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -83,8 +83,16 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +114,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -151,7 +165,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -244,6 +258,8 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1434,57 +1450,57 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -1508,37 +1524,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>32.76053524292911</v>
+        <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>129.4325986170056</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>207.0727386268931</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>243.9802655280589</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>241.6601110204685</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>207.1396449035606</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>153.0315282935943</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>153.0315282935943</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>153.0315282935943</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>153.0315282935943</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>153.0315282935943</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1890,7 +1906,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>765.1576414679723</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -2119,7 +2135,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>191.2894103669931</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -2194,7 +2210,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>420.8367028073848</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -3208,57 +3224,57 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="L12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -3282,37 +3298,37 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>9.785888920321048</v>
+        <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>46.1742513621563</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>91.90205973843209</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>149.7391847266321</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>216.3111720417033</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>292.7414325310211</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
-        <v>358.5648409233147</v>
+        <v>0</v>
       </c>
       <c r="L13" s="39" t="n">
-        <v>429.5676106826317</v>
+        <v>0</v>
       </c>
       <c r="M13" s="39" t="n">
-        <v>489.5432484211076</v>
+        <v>0</v>
       </c>
       <c r="N13" s="39" t="n">
-        <v>536.5221375252406</v>
+        <v>0</v>
       </c>
       <c r="O13" s="39" t="n">
-        <v>568.4393062135854</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3664,7 +3680,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>32.61962973440349</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -3893,7 +3909,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>16.30981486720174</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -3968,7 +3984,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>6.523925946880698</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5030,32 +5046,32 @@
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="I12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J12" s="39" t="inlineStr">
         <is>
-          <t>increase debt</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="39" t="inlineStr">
@@ -5104,22 +5120,22 @@
         <v>0</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>188.1442257170714</v>
+        <v>0</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>321.726759825858</v>
+        <v>0</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>389.0185416170291</v>
+        <v>0</v>
       </c>
       <c r="H13" s="39" t="n">
-        <v>392.5065467157357</v>
+        <v>0</v>
       </c>
       <c r="I13" s="39" t="n">
-        <v>224.9243005734117</v>
+        <v>0</v>
       </c>
       <c r="J13" s="39" t="n">
-        <v>12.42614874820384</v>
+        <v>0</v>
       </c>
       <c r="K13" s="39" t="n">
         <v>0</v>
@@ -5284,7 +5300,7 @@
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="E16" s="33" t="n">
         <v>0</v>
@@ -5299,22 +5315,22 @@
         <v>0</v>
       </c>
       <c r="I16" s="33" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="J16" s="33" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="K16" s="33" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="L16" s="33" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="M16" s="33" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="N16" s="33" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="O16" s="33" t="n">
         <v>0</v>
@@ -5486,7 +5502,7 @@
         </is>
       </c>
       <c r="C19" s="32" t="n">
-        <v>783.624304073695</v>
+        <v>0</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
@@ -5715,7 +5731,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>156.724860814739</v>
+        <v>0</v>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
@@ -5790,7 +5806,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>391.8121520368475</v>
+        <v>0</v>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
@@ -5865,7 +5881,7 @@
         </is>
       </c>
       <c r="C24" s="33" t="n">
-        <v>745</v>
+        <v>100</v>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
@@ -5940,7 +5956,7 @@
         </is>
       </c>
       <c r="C25" s="32" t="n">
-        <v>16</v>
+        <v>13.45271494470075</v>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>

</xml_diff>